<commit_message>
Publish the application documents, keep the working notes out of the repo
The 2027 application (programme description, form answers, budget, work
plan, team text and their PDF/DOCX/XLSX builds) is deliberately public.
The internal working notes (things to confirm, evidence list, submission
checklist, sources, validation record, package overview) are not: they
stay on disk and behind Cloudflare Access, and are now gitignored.

The dossier reader no longer links to them. A follow-up history rewrite
removes their earlier committed copies.

Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/prijava/03-troskovnik-i-plan-financiranja.xlsx
+++ b/prijava/03-troskovnik-i-plan-financiranja.xlsx
@@ -13,7 +13,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Kontrola" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm.Print_Area" localSheetId="0">'Troškovnik'!$A$1:$J$17</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="0">'Troškovnik'!$A$1:$J$18</definedName>
     <definedName name="_xlnm.Print_Area" localSheetId="1">'Plan financiranja'!$A$1:$D$6</definedName>
   </definedNames>
   <calcPr calcId="124519" calcMode="auto" fullCalcOnLoad="1" forceFullCalc="1"/>
@@ -562,7 +562,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:J17"/>
+  <dimension ref="A1:J18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="7" customWidth="1" min="1" max="1"/>
@@ -587,7 +587,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Portal otvorenih podataka Hrvatskog audiovizualnog centra</t>
+          <t>Sredstva: otvoreni registar javnog financiranja audiovizualnih djelatnosti</t>
         </is>
       </c>
     </row>
@@ -656,21 +656,21 @@
       </c>
       <c r="B5" s="6" t="inlineStr">
         <is>
-          <t>Honorari suradnika</t>
+          <t>Plaće, autorski honorari i intelektualne usluge</t>
         </is>
       </c>
       <c r="C5" s="6" t="inlineStr">
         <is>
-          <t>Primarna ručna provjera zapisa</t>
+          <t>Honorari suradnika: istraživači-redaktori, primarna urednička provjera svakog zapisa prema izvornom dokumentu</t>
         </is>
       </c>
       <c r="D5" s="6" t="inlineStr">
         <is>
-          <t>40 radnih dana × 125 EUR</t>
+          <t>32 radna dana × 125 EUR</t>
         </is>
       </c>
       <c r="E5" s="5" t="n">
-        <v>40</v>
+        <v>32</v>
       </c>
       <c r="F5" s="6" t="inlineStr">
         <is>
@@ -680,12 +680,11 @@
       <c r="G5" s="7" t="n">
         <v>125</v>
       </c>
-      <c r="H5" s="7">
-        <f>E5*G5</f>
-        <v/>
+      <c r="H5" s="7" t="n">
+        <v>4000</v>
       </c>
       <c r="I5" s="7" t="n">
-        <v>5000</v>
+        <v>4000</v>
       </c>
       <c r="J5" s="7" t="n">
         <v>0</v>
@@ -697,21 +696,21 @@
       </c>
       <c r="B6" s="9" t="inlineStr">
         <is>
-          <t>Honorari suradnika</t>
+          <t>Plaće, autorski honorari i intelektualne usluge</t>
         </is>
       </c>
       <c r="C6" s="9" t="inlineStr">
         <is>
-          <t>Istraživanje i pribavljanje nedostajućih izvora</t>
+          <t>Honorari suradnika: istraživanje i pribavljanje nedostupnih izvora, unos novopronađenih dokumenata i evidentiranje sjedišta korisnika</t>
         </is>
       </c>
       <c r="D6" s="9" t="inlineStr">
         <is>
-          <t>12 radnih dana × 125 EUR</t>
+          <t>8 radnih dana × 125 EUR</t>
         </is>
       </c>
       <c r="E6" s="8" t="n">
-        <v>12</v>
+        <v>8</v>
       </c>
       <c r="F6" s="9" t="inlineStr">
         <is>
@@ -721,12 +720,11 @@
       <c r="G6" s="10" t="n">
         <v>125</v>
       </c>
-      <c r="H6" s="10">
-        <f>E6*G6</f>
-        <v/>
+      <c r="H6" s="10" t="n">
+        <v>1000</v>
       </c>
       <c r="I6" s="10" t="n">
-        <v>1500</v>
+        <v>1000</v>
       </c>
       <c r="J6" s="10" t="n">
         <v>0</v>
@@ -738,21 +736,21 @@
       </c>
       <c r="B7" s="6" t="inlineStr">
         <is>
-          <t>Honorari suradnika</t>
+          <t>Plaće, autorski honorari i intelektualne usluge</t>
         </is>
       </c>
       <c r="C7" s="6" t="inlineStr">
         <is>
-          <t>Drugi pregled ispravaka i kontrolni uzorak</t>
+          <t>Honorari suradnika: drugi pregled izmijenjenih i nerazriješenih zapisa i kontrolni uzorak 10 %</t>
         </is>
       </c>
       <c r="D7" s="6" t="inlineStr">
         <is>
-          <t>8 radnih dana × 125 EUR</t>
+          <t>6 radnih dana × 125 EUR</t>
         </is>
       </c>
       <c r="E7" s="5" t="n">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="F7" s="6" t="inlineStr">
         <is>
@@ -762,12 +760,11 @@
       <c r="G7" s="7" t="n">
         <v>125</v>
       </c>
-      <c r="H7" s="7">
-        <f>E7*G7</f>
-        <v/>
+      <c r="H7" s="7" t="n">
+        <v>750</v>
       </c>
       <c r="I7" s="7" t="n">
-        <v>1000</v>
+        <v>750</v>
       </c>
       <c r="J7" s="7" t="n">
         <v>0</v>
@@ -779,39 +776,38 @@
       </c>
       <c r="B8" s="9" t="inlineStr">
         <is>
-          <t>Plaće</t>
+          <t>Plaće, autorski honorari i intelektualne usluge</t>
         </is>
       </c>
       <c r="C8" s="9" t="inlineStr">
         <is>
-          <t>Voditelj, urednik podataka i arhitekt sustava</t>
+          <t>Autorski honorari: četiri tematske analize vanjskih autora (800–1.500 riječi; autorskim ugovorom prenosi se pravo objave na portalu, HR/EN, i u godišnjem pregledu)</t>
         </is>
       </c>
       <c r="D8" s="9" t="inlineStr">
         <is>
-          <t>160 sati × 25 EUR razmjernog bruto troška</t>
+          <t>4 autorska teksta × 200 EUR</t>
         </is>
       </c>
       <c r="E8" s="8" t="n">
-        <v>160</v>
+        <v>4</v>
       </c>
       <c r="F8" s="9" t="inlineStr">
         <is>
-          <t>sat</t>
+          <t>autorski tekst</t>
         </is>
       </c>
       <c r="G8" s="10" t="n">
-        <v>25</v>
-      </c>
-      <c r="H8" s="10">
-        <f>E8*G8</f>
-        <v/>
+        <v>200</v>
+      </c>
+      <c r="H8" s="10" t="n">
+        <v>800</v>
       </c>
       <c r="I8" s="10" t="n">
+        <v>800</v>
+      </c>
+      <c r="J8" s="10" t="n">
         <v>0</v>
-      </c>
-      <c r="J8" s="10" t="n">
-        <v>4000</v>
       </c>
     </row>
     <row r="9" ht="42" customHeight="1">
@@ -820,39 +816,38 @@
       </c>
       <c r="B9" s="6" t="inlineStr">
         <is>
-          <t>Online sustavi i tehnički troškovi</t>
+          <t>Plaće, autorski honorari i intelektualne usluge</t>
         </is>
       </c>
       <c r="C9" s="6" t="inlineStr">
         <is>
-          <t>Hosting i izvršavanje javnog portala</t>
+          <t>Plaća: urednik i voditelj programa (uređivanje izdanja i autorski tekstovi, metodologija, obuka i nadzor suradnika, odluke o spornim zapisima, objava izdanja), razmjerni bruto trošak</t>
         </is>
       </c>
       <c r="D9" s="6" t="inlineStr">
         <is>
-          <t>12 mjeseci × 15 EUR</t>
+          <t>160 sati × 25 EUR</t>
         </is>
       </c>
       <c r="E9" s="5" t="n">
-        <v>12</v>
+        <v>160</v>
       </c>
       <c r="F9" s="6" t="inlineStr">
         <is>
-          <t>mjesec</t>
+          <t>sat</t>
         </is>
       </c>
       <c r="G9" s="7" t="n">
-        <v>15</v>
-      </c>
-      <c r="H9" s="7">
-        <f>E9*G9</f>
-        <v/>
+        <v>25</v>
+      </c>
+      <c r="H9" s="7" t="n">
+        <v>4000</v>
       </c>
       <c r="I9" s="7" t="n">
         <v>0</v>
       </c>
       <c r="J9" s="7" t="n">
-        <v>180</v>
+        <v>4000</v>
       </c>
     </row>
     <row r="10" ht="42" customHeight="1">
@@ -861,39 +856,38 @@
       </c>
       <c r="B10" s="9" t="inlineStr">
         <is>
-          <t>Online sustavi i tehnički troškovi</t>
+          <t>Plaće, autorski honorari i intelektualne usluge</t>
         </is>
       </c>
       <c r="C10" s="9" t="inlineStr">
         <is>
-          <t>Pohrana izvora i sigurnosne kopije</t>
+          <t>Intelektualne usluge: provjera licenci i priprema paketa za ponovnu uporabu</t>
         </is>
       </c>
       <c r="D10" s="9" t="inlineStr">
         <is>
-          <t>12 mjeseci × 5 EUR</t>
+          <t>1 × 80 EUR (paušalno)</t>
         </is>
       </c>
       <c r="E10" s="8" t="n">
-        <v>12</v>
+        <v>1</v>
       </c>
       <c r="F10" s="9" t="inlineStr">
         <is>
-          <t>mjesec</t>
+          <t>paket</t>
         </is>
       </c>
       <c r="G10" s="10" t="n">
-        <v>5</v>
-      </c>
-      <c r="H10" s="10">
-        <f>E10*G10</f>
-        <v/>
+        <v>80</v>
+      </c>
+      <c r="H10" s="10" t="n">
+        <v>80</v>
       </c>
       <c r="I10" s="10" t="n">
         <v>0</v>
       </c>
       <c r="J10" s="10" t="n">
-        <v>60</v>
+        <v>80</v>
       </c>
     </row>
     <row r="11" ht="42" customHeight="1">
@@ -902,17 +896,17 @@
       </c>
       <c r="B11" s="6" t="inlineStr">
         <is>
-          <t>Online sustavi i tehnički troškovi</t>
+          <t>Prijevod i lektura, priprema, grafičko oblikovanje</t>
         </is>
       </c>
       <c r="C11" s="6" t="inlineStr">
         <is>
-          <t>Domena i DNS usluge</t>
+          <t>Lektura hrvatskih tekstova: tematske analize, metodološke bilješke i godišnji pregled (oko 50 kartica; pregledi rokova i uredničke bilješke lektoriraju se u uredništvu), prijevod na engleski (oko 17 kartica) i grafičko oblikovanje godišnjeg pregleda (PDF)</t>
         </is>
       </c>
       <c r="D11" s="6" t="inlineStr">
         <is>
-          <t>godišnji trošak</t>
+          <t>1 × 550 EUR (paušalno)</t>
         </is>
       </c>
       <c r="E11" s="5" t="n">
@@ -920,21 +914,20 @@
       </c>
       <c r="F11" s="6" t="inlineStr">
         <is>
-          <t>godina</t>
+          <t>paket</t>
         </is>
       </c>
       <c r="G11" s="7" t="n">
-        <v>20</v>
-      </c>
-      <c r="H11" s="7">
-        <f>E11*G11</f>
-        <v/>
+        <v>550</v>
+      </c>
+      <c r="H11" s="7" t="n">
+        <v>550</v>
       </c>
       <c r="I11" s="7" t="n">
+        <v>550</v>
+      </c>
+      <c r="J11" s="7" t="n">
         <v>0</v>
-      </c>
-      <c r="J11" s="7" t="n">
-        <v>20</v>
       </c>
     </row>
     <row r="12" ht="42" customHeight="1">
@@ -943,39 +936,38 @@
       </c>
       <c r="B12" s="9" t="inlineStr">
         <is>
-          <t>Online sustavi i tehnički troškovi</t>
+          <t>Prezentacija i promocija programa</t>
         </is>
       </c>
       <c r="C12" s="9" t="inlineStr">
         <is>
-          <t>Nužni OCR/API alati za obradu iznimaka</t>
+          <t>Dva javna predstavljanja izdanja, jedno izvan Zagreba, u prostorima ustanova domaćina bez najma (putni trošak, oprema, jednostrani tiskani materijal)</t>
         </is>
       </c>
       <c r="D12" s="9" t="inlineStr">
         <is>
-          <t>ograničeni godišnji paket</t>
+          <t>2 predstavljanja × 200 EUR</t>
         </is>
       </c>
       <c r="E12" s="8" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F12" s="9" t="inlineStr">
         <is>
-          <t>paket</t>
+          <t>predstavljanje</t>
         </is>
       </c>
       <c r="G12" s="10" t="n">
-        <v>40</v>
-      </c>
-      <c r="H12" s="10">
-        <f>E12*G12</f>
-        <v/>
+        <v>200</v>
+      </c>
+      <c r="H12" s="10" t="n">
+        <v>400</v>
       </c>
       <c r="I12" s="10" t="n">
+        <v>400</v>
+      </c>
+      <c r="J12" s="10" t="n">
         <v>0</v>
-      </c>
-      <c r="J12" s="10" t="n">
-        <v>40</v>
       </c>
     </row>
     <row r="13" ht="42" customHeight="1">
@@ -984,39 +976,38 @@
       </c>
       <c r="B13" s="6" t="inlineStr">
         <is>
-          <t>Administracija i primopredaja</t>
+          <t>Uredski troškovi</t>
         </is>
       </c>
       <c r="C13" s="6" t="inlineStr">
         <is>
-          <t>Razmjerni računovodstveni trošak programa</t>
+          <t>Poslužiteljske usluge (smještaj i rad portala), pohrana izvornika i sigurnosnih kopija, domena i DNS (12 mjeseci)</t>
         </is>
       </c>
       <c r="D13" s="6" t="inlineStr">
         <is>
-          <t>12 mjeseci × 10 EUR</t>
+          <t>12 mjeseci, 260 EUR godišnje</t>
         </is>
       </c>
       <c r="E13" s="5" t="n">
-        <v>12</v>
+        <v>1</v>
       </c>
       <c r="F13" s="6" t="inlineStr">
         <is>
-          <t>mjesec</t>
+          <t>godina</t>
         </is>
       </c>
       <c r="G13" s="7" t="n">
-        <v>10</v>
-      </c>
-      <c r="H13" s="7">
-        <f>E13*G13</f>
-        <v/>
+        <v>260</v>
+      </c>
+      <c r="H13" s="7" t="n">
+        <v>260</v>
       </c>
       <c r="I13" s="7" t="n">
         <v>0</v>
       </c>
       <c r="J13" s="7" t="n">
-        <v>120</v>
+        <v>260</v>
       </c>
     </row>
     <row r="14" ht="42" customHeight="1">
@@ -1025,17 +1016,17 @@
       </c>
       <c r="B14" s="9" t="inlineStr">
         <is>
-          <t>Administracija i primopredaja</t>
+          <t>Uredski troškovi</t>
         </is>
       </c>
       <c r="C14" s="9" t="inlineStr">
         <is>
-          <t>Provjera licenci i priprema završnog paketa</t>
+          <t>Alati za strojno čitanje skeniranih dokumenata (OCR)</t>
         </is>
       </c>
       <c r="D14" s="9" t="inlineStr">
         <is>
-          <t>projektni paket</t>
+          <t>1 × 40 EUR (paušalno)</t>
         </is>
       </c>
       <c r="E14" s="8" t="n">
@@ -1047,46 +1038,82 @@
         </is>
       </c>
       <c r="G14" s="10" t="n">
-        <v>80</v>
-      </c>
-      <c r="H14" s="10">
-        <f>E14*G14</f>
-        <v/>
+        <v>40</v>
+      </c>
+      <c r="H14" s="10" t="n">
+        <v>40</v>
       </c>
       <c r="I14" s="10" t="n">
         <v>0</v>
       </c>
       <c r="J14" s="10" t="n">
-        <v>80</v>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" s="11" t="inlineStr">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="15" ht="42" customHeight="1">
+      <c r="A15" s="5" t="n">
+        <v>11</v>
+      </c>
+      <c r="B15" s="6" t="inlineStr">
+        <is>
+          <t>Uredski troškovi</t>
+        </is>
+      </c>
+      <c r="C15" s="6" t="inlineStr">
+        <is>
+          <t>Razmjerni računovodstveni trošak programa</t>
+        </is>
+      </c>
+      <c r="D15" s="6" t="inlineStr">
+        <is>
+          <t>12 mjeseci × 10 EUR</t>
+        </is>
+      </c>
+      <c r="E15" s="5" t="n">
+        <v>12</v>
+      </c>
+      <c r="F15" s="6" t="inlineStr">
+        <is>
+          <t>mjesec</t>
+        </is>
+      </c>
+      <c r="G15" s="7" t="n">
+        <v>10</v>
+      </c>
+      <c r="H15" s="7" t="n">
+        <v>120</v>
+      </c>
+      <c r="I15" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="J15" s="7" t="n">
+        <v>120</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="11" t="inlineStr">
         <is>
           <t>UKUPNO</t>
         </is>
       </c>
-      <c r="B15" s="11" t="n"/>
-      <c r="C15" s="11" t="n"/>
-      <c r="D15" s="11" t="n"/>
-      <c r="E15" s="11" t="n"/>
-      <c r="F15" s="11" t="n"/>
-      <c r="G15" s="11" t="n"/>
-      <c r="H15" s="12">
-        <f>SUM(H5:H14)</f>
-        <v/>
-      </c>
-      <c r="I15" s="12">
-        <f>SUM(I5:I14)</f>
-        <v/>
-      </c>
-      <c r="J15" s="12">
-        <f>SUM(J5:J14)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="17" ht="32" customHeight="1">
-      <c r="A17" s="13" t="inlineStr">
+      <c r="B16" s="11" t="n"/>
+      <c r="C16" s="11" t="n"/>
+      <c r="D16" s="11" t="n"/>
+      <c r="E16" s="11" t="n"/>
+      <c r="F16" s="11" t="n"/>
+      <c r="G16" s="11" t="n"/>
+      <c r="H16" s="12" t="n">
+        <v>12000</v>
+      </c>
+      <c r="I16" s="12" t="n">
+        <v>7500</v>
+      </c>
+      <c r="J16" s="12" t="n">
+        <v>4500</v>
+      </c>
+    </row>
+    <row r="18" ht="32" customHeight="1">
+      <c r="A18" s="13" t="inlineStr">
         <is>
           <t>Napomena: troškovnik obuhvaća samo rad i troškove nastale tijekom 2027. Postojeći razvoj iz 2026. ne traži se retroaktivno.</t>
         </is>
@@ -1095,16 +1122,16 @@
   </sheetData>
   <mergeCells count="5">
     <mergeCell ref="A1:J1"/>
-    <mergeCell ref="A17:J17"/>
+    <mergeCell ref="A18:J18"/>
     <mergeCell ref="A3:J3"/>
-    <mergeCell ref="A15:G15"/>
+    <mergeCell ref="A16:G16"/>
     <mergeCell ref="A2:J2"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup orientation="landscape" paperSize="9" fitToHeight="1" fitToWidth="1"/>
   <headerFooter>
     <oddHeader/>
-    <oddFooter>&amp;CPortal otvorenih podataka Hrvatskog audiovizualnog centra&amp;RStranica &amp;P od &amp;N</oddFooter>
+    <oddFooter>&amp;CSredstva: otvoreni registar javnog financiranja audiovizualnih djelatnosti&amp;RStranica &amp;P od &amp;N</oddFooter>
     <evenHeader/>
     <evenFooter/>
     <firstHeader/>
@@ -1183,7 +1210,7 @@
       </c>
       <c r="B5" s="16" t="inlineStr">
         <is>
-          <t>vlastita sredstva/rad</t>
+          <t>vlastita sredstva i razmjerni trošak rada u 2027.</t>
         </is>
       </c>
       <c r="C5" s="17" t="n">
@@ -1200,13 +1227,11 @@
         </is>
       </c>
       <c r="B6" s="19" t="inlineStr"/>
-      <c r="C6" s="20">
-        <f>SUM(C4:C5)</f>
-        <v/>
-      </c>
-      <c r="D6" s="21">
-        <f>SUM(D4:D5)</f>
-        <v/>
+      <c r="C6" s="20" t="n">
+        <v>12000</v>
+      </c>
+      <c r="D6" s="21" t="n">
+        <v>1</v>
       </c>
     </row>
   </sheetData>
@@ -1246,72 +1271,72 @@
     <row r="2" ht="55" customHeight="1">
       <c r="A2" s="23" t="inlineStr">
         <is>
-          <t>Primarna ručna provjera</t>
+          <t>Honorari suradnika (istraživači-redaktori)</t>
         </is>
       </c>
       <c r="B2" s="23" t="inlineStr">
         <is>
-          <t>Usporedba svakog zapisa završne baze s izvornim dokumentom: iznos, valuta, godina, rok, kategorija, naziv projekta, korisnik i status financiranja.</t>
+          <t>Primarna urednička provjera svakog zapisa prema izvornom dokumentu u sedam polja (naziv projekta, korisnik i imenovani autori, program, godina i rok, iznos i valuta, status financiranja, poveznica na izvor); istraživanje i pribavljanje izvora koji više nisu dostupni na mreži uz evidentiranje sjedišta korisnika; drugi pregled svih izmijenjenih i nerazriješenih zapisa te kontrolni uzorak od najmanje 10 %. Jedinična cijena 125,00 EUR po radnom danu iskazana je kao ukupni trošak podnositelja; 46 radnih dana raspoređeno je na dvoje suradnika kroz devet mjeseci.</t>
         </is>
       </c>
     </row>
     <row r="3" ht="55" customHeight="1">
       <c r="A3" s="23" t="inlineStr">
         <is>
-          <t>Istraživanje izvora</t>
+          <t>Autorski honorari</t>
         </is>
       </c>
       <c r="B3" s="23" t="inlineStr">
         <is>
-          <t>Usporedba korpusa sa službenim objavama, pronalaženje neaktivnih poveznica, priprema popisa građe koja se traži od HAVC-a te unos novopronađenih dokumenata.</t>
+          <t>Četiri tematske analize vanjskih autora (800–1.500 riječi, s tablicama i engleskim sažetkom); autorskim ugovorom prenosi se pravo objave na portalu (HR/EN) i u godišnjem pregledu.</t>
         </is>
       </c>
     </row>
     <row r="4" ht="55" customHeight="1">
       <c r="A4" s="23" t="inlineStr">
         <is>
-          <t>Drugi pregled i QA</t>
+          <t>Plaća urednika</t>
         </is>
       </c>
       <c r="B4" s="23" t="inlineStr">
         <is>
-          <t>Neovisna provjera svih ispravljenih i nerazriješenih zapisa te najmanje 10% nasumično odabranih zapisa koji nisu mijenjani.</t>
+          <t>Uređivanje dvanaest izdanja i autorski tekstovi, metodologija i shema, obuka i nadzor suradnika, odluke o spornim zapisima, objava izdanja. Iskazano je 160 sati razmjernog bruto troška plaće u 2027.; rad iznad tog opsega Aning Film osigurava izvan troškovnika.</t>
         </is>
       </c>
     </row>
     <row r="5" ht="55" customHeight="1">
       <c r="A5" s="23" t="inlineStr">
         <is>
-          <t>Voditelj programa</t>
+          <t>Prijevod i lektura, grafičko oblikovanje</t>
         </is>
       </c>
       <c r="B5" s="23" t="inlineStr">
         <is>
-          <t>Metodologija, shema, alat za provjeru, obuka i nadzor suradnika, uredničke odluke, validacija, objava i završna primopredaja. Samo rad tijekom 2027.</t>
+          <t>Lektura tematskih analiza, metodoloških bilježaka i godišnjeg pregleda (oko 50 kartica; pregledi rokova i uredničke bilješke lektoriraju se u uredništvu), prijevod sažetaka i godišnjeg pregleda na engleski (oko 17 kartica) i grafičko oblikovanje godišnjeg pregleda u PDF-u.</t>
         </is>
       </c>
     </row>
     <row r="6" ht="55" customHeight="1">
       <c r="A6" s="23" t="inlineStr">
         <is>
-          <t>Online sustavi</t>
+          <t>Prezentacija i promocija</t>
         </is>
       </c>
       <c r="B6" s="23" t="inlineStr">
         <is>
-          <t>Hosting, pohrana, sigurnosne kopije, domena i nužni OCR/API alati izravno vezani uz provedbu.</t>
+          <t>Dva javna predstavljanja izdanja tijekom 2027., jedno u Zagrebu i jedno izvan Zagreba, u prostorima ustanova domaćina bez najma: putni trošak, oprema i jednostrani tiskani materijal.</t>
         </is>
       </c>
     </row>
     <row r="7" ht="55" customHeight="1">
       <c r="A7" s="23" t="inlineStr">
         <is>
-          <t>Administracija</t>
+          <t>Uredski troškovi</t>
         </is>
       </c>
       <c r="B7" s="23" t="inlineStr">
         <is>
-          <t>Razmjerni računovodstveni trošak, provjera otvorenih licenci i priprema urednog završnog paketa za HAVC.</t>
+          <t>Poslužiteljske usluge (smještaj i rad portala), pohrana izvornika i sigurnosnih kopija, domena i DNS, alati za strojno čitanje skeniranih dokumenata (OCR), razmjerni računovodstveni trošak te provjera licenci i priprema paketa za ponovnu uporabu. Razvoj iz 2026. nije uračunat.</t>
         </is>
       </c>
     </row>
@@ -1352,7 +1377,7 @@
         </is>
       </c>
       <c r="B2" s="25">
-        <f>'Troškovnik'!H15</f>
+        <f>'Troškovnik'!H16</f>
         <v/>
       </c>
     </row>
@@ -1363,7 +1388,7 @@
         </is>
       </c>
       <c r="B3" s="25">
-        <f>'Troškovnik'!I15</f>
+        <f>'Troškovnik'!I16</f>
         <v/>
       </c>
     </row>
@@ -1374,7 +1399,7 @@
         </is>
       </c>
       <c r="B4" s="25">
-        <f>'Troškovnik'!J15</f>
+        <f>'Troškovnik'!J16</f>
         <v/>
       </c>
     </row>

</xml_diff>